<commit_message>
Updated Blattabacterium host genome referencing
</commit_message>
<xml_diff>
--- a/data/Blattabacterium/Blattabacterium_genome-data.xlsx
+++ b/data/Blattabacterium/Blattabacterium_genome-data.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/Documents/Zhuzhi genomes/HGT/Blattabacterium_refs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/PostDoc/HGT_pipeline/data/Blattabacterium/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{654F1CDD-E0DA-8B4F-83DB-4B89CA542591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74F289EB-2BE7-3A49-AEFD-352BAE5EDABC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2260" yWindow="1480" windowWidth="33400" windowHeight="26520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11440" yWindow="1440" windowWidth="17360" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="167">
   <si>
     <t>#</t>
   </si>
@@ -491,13 +491,43 @@
   </si>
   <si>
     <t>Kambhampati et al. Complete genome sequence of the endosymbiont Blattabacterium from the cockroach Nauphoeta cinerea (Blattodea: Blaberidae). Genomics 102 (5-6), 479-483 (2013)</t>
+  </si>
+  <si>
+    <t>Used for aging?</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Diploptera punctata</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Wasn't included in initial Blattabacterium chunk alignment step</t>
+  </si>
+  <si>
+    <t>CP049785.1</t>
+  </si>
+  <si>
+    <t>NCBI</t>
+  </si>
+  <si>
+    <t>Panesthia cribrata</t>
+  </si>
+  <si>
+    <t>Panesthia lata</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -546,8 +576,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -558,6 +596,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -584,7 +628,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -611,6 +655,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -831,17 +881,17 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D98"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:F92"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.6640625" style="2"/>
     <col min="2" max="2" width="21.5" style="2" customWidth="1"/>
-    <col min="3" max="3" width="16.1640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="195" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.83203125" style="2" customWidth="1"/>
     <col min="5" max="16384" width="12.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -854,8 +904,14 @@
       <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E1" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -868,8 +924,11 @@
       <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E2" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" customHeight="1">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -882,8 +941,11 @@
       <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E3" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -896,8 +958,11 @@
       <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E4" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" customHeight="1">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -910,8 +975,11 @@
       <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E5" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -924,8 +992,11 @@
       <c r="D6" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E6" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -938,8 +1009,11 @@
       <c r="D7" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E7" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" customHeight="1">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -952,8 +1026,11 @@
       <c r="D8" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E8" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -966,8 +1043,11 @@
       <c r="D9" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E9" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" customHeight="1">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -980,8 +1060,11 @@
       <c r="D10" s="3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E10" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" customHeight="1">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -994,8 +1077,11 @@
       <c r="D11" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E11" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" customHeight="1">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1008,8 +1094,11 @@
       <c r="D12" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E12" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" customHeight="1">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1022,8 +1111,11 @@
       <c r="D13" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E13" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" customHeight="1">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1036,8 +1128,11 @@
       <c r="D14" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E14" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15.75" customHeight="1">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1050,8 +1145,11 @@
       <c r="D15" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E15" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.75" customHeight="1">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1064,8 +1162,11 @@
       <c r="D16" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E16" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15.75" customHeight="1">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1078,8 +1179,11 @@
       <c r="D17" s="3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E17" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15.75" customHeight="1">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1092,8 +1196,11 @@
       <c r="D18" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E18" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" customHeight="1">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1106,8 +1213,11 @@
       <c r="D19" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E19" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" customHeight="1">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1120,8 +1230,11 @@
       <c r="D20" s="3" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E20" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15.75" customHeight="1">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1134,8 +1247,11 @@
       <c r="D21" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E21" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1148,8 +1264,11 @@
       <c r="D22" s="3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E22" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15.75" customHeight="1">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1162,8 +1281,11 @@
       <c r="D23" s="3" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E23" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" customHeight="1">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1176,8 +1298,11 @@
       <c r="D24" s="3" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E24" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15.75" customHeight="1">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1190,8 +1315,11 @@
       <c r="D25" s="3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E25" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" customHeight="1">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1204,8 +1332,11 @@
       <c r="D26" s="3" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E26" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" customHeight="1">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1218,8 +1349,11 @@
       <c r="D27" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E27" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" customHeight="1">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1232,8 +1366,11 @@
       <c r="D28" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E28" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -1246,8 +1383,11 @@
       <c r="D29" s="3" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E29" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -1260,8 +1400,11 @@
       <c r="D30" s="3" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E30" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -1274,8 +1417,11 @@
       <c r="D31" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E31" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -1288,8 +1434,11 @@
       <c r="D32" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E32" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" customHeight="1">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1302,8 +1451,11 @@
       <c r="D33" s="3" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E33" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" customHeight="1">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1316,8 +1468,11 @@
       <c r="D34" s="3" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E34" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="15.75" customHeight="1">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1330,8 +1485,11 @@
       <c r="D35" s="3" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E35" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" customHeight="1">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1344,8 +1502,11 @@
       <c r="D36" s="3" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E36" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="15.75" customHeight="1">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -1358,8 +1519,11 @@
       <c r="D37" s="3" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E37" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="15.75" customHeight="1">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -1372,8 +1536,11 @@
       <c r="D38" s="3" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E38" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="15.75" customHeight="1">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -1386,8 +1553,11 @@
       <c r="D39" s="3" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E39" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="15.75" customHeight="1">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -1400,8 +1570,11 @@
       <c r="D40" s="3" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E40" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" customHeight="1">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -1414,8 +1587,11 @@
       <c r="D41" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E41" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="15.75" customHeight="1">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -1428,8 +1604,11 @@
       <c r="D42" s="3" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E42" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="15.75" customHeight="1">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -1442,8 +1621,11 @@
       <c r="D43" s="3" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E43" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="15.75" customHeight="1">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -1456,8 +1638,11 @@
       <c r="D44" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E44" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="15.75" customHeight="1">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -1470,8 +1655,11 @@
       <c r="D45" s="3" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E45" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="15.75" customHeight="1">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -1484,8 +1672,11 @@
       <c r="D46" s="3" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E46" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="15.75" customHeight="1">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -1498,8 +1689,11 @@
       <c r="D47" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E47" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="15.75" customHeight="1">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -1512,8 +1706,11 @@
       <c r="D48" s="7" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E48" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="15.75" customHeight="1">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -1526,8 +1723,11 @@
       <c r="D49" s="7" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E49" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="15.75" customHeight="1">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -1540,8 +1740,11 @@
       <c r="D50" s="7" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E50" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="15.75" customHeight="1">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -1554,8 +1757,11 @@
       <c r="D51" s="7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E51" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="15.75" customHeight="1">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -1568,8 +1774,11 @@
       <c r="D52" s="7" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E52" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="15.75" customHeight="1">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -1582,8 +1791,11 @@
       <c r="D53" s="7" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E53" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="15.75" customHeight="1">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -1596,8 +1808,11 @@
       <c r="D54" s="7" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E54" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="15.75" customHeight="1">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -1610,8 +1825,11 @@
       <c r="D55" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E55" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="15.75" customHeight="1">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -1624,8 +1842,11 @@
       <c r="D56" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E56" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="15.75" customHeight="1">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -1638,8 +1859,11 @@
       <c r="D57" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E57" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="15.75" customHeight="1">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -1652,8 +1876,11 @@
       <c r="D58" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E58" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="15.75" customHeight="1">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -1666,8 +1893,11 @@
       <c r="D59" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E59" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="15.75" customHeight="1">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -1680,8 +1910,11 @@
       <c r="D60" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E60" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="15.75" customHeight="1">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -1694,8 +1927,11 @@
       <c r="D61" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E61" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="15.75" customHeight="1">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -1708,8 +1944,11 @@
       <c r="D62" s="7" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E62" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="15.75" customHeight="1">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -1722,8 +1961,11 @@
       <c r="D63" s="7" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E63" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="15.75" customHeight="1">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -1736,8 +1978,11 @@
       <c r="D64" s="7" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E64" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="15.75" customHeight="1">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -1750,8 +1995,11 @@
       <c r="D65" s="7" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E65" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="15.75" customHeight="1">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -1764,8 +2012,11 @@
       <c r="D66" s="7" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E66" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="15.75" customHeight="1">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -1778,8 +2029,11 @@
       <c r="D67" s="7" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E67" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="15.75" customHeight="1">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -1792,8 +2046,11 @@
       <c r="D68" s="7" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E68" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="15.75" customHeight="1">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -1806,8 +2063,11 @@
       <c r="D69" s="7" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E69" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="15.75" customHeight="1">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -1820,8 +2080,11 @@
       <c r="D70" s="7" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E70" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="15.75" customHeight="1">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -1834,8 +2097,11 @@
       <c r="D71" s="8" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E71" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="15.75" customHeight="1">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -1848,8 +2114,11 @@
       <c r="D72" s="8" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E72" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="15.75" customHeight="1">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -1862,8 +2131,11 @@
       <c r="D73" s="7" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E73" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="15.75" customHeight="1">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -1876,8 +2148,11 @@
       <c r="D74" s="7" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E74" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="15.75" customHeight="1">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -1890,8 +2165,11 @@
       <c r="D75" s="7" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E75" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="15.75" customHeight="1">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -1904,8 +2182,11 @@
       <c r="D76" s="7" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E76" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="15.75" customHeight="1">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -1918,8 +2199,11 @@
       <c r="D77" s="2" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E77" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="15.75" customHeight="1">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -1932,48 +2216,85 @@
       <c r="D78" s="7" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C79" s="7"/>
-      <c r="D79" s="7"/>
-    </row>
-    <row r="87" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E78" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A79" s="11"/>
+      <c r="B79" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F79" s="7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A80" s="11"/>
+      <c r="B80" s="11"/>
+      <c r="C80" s="11"/>
+      <c r="D80" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E80" s="11"/>
+      <c r="F80" s="7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A81" s="11"/>
+      <c r="B81" s="11"/>
+      <c r="C81" s="11"/>
+      <c r="D81" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="E81" s="11"/>
+      <c r="F81" s="7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="15.75" customHeight="1">
+      <c r="B82" s="7"/>
+      <c r="C82" s="7"/>
+    </row>
+    <row r="83" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C83" s="7"/>
+    </row>
+    <row r="84" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C84" s="7"/>
+    </row>
+    <row r="85" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C85" s="7"/>
+    </row>
+    <row r="86" spans="1:6" ht="15.75" customHeight="1">
+      <c r="C86" s="7"/>
+    </row>
+    <row r="87" spans="1:6" ht="15.75" customHeight="1">
       <c r="C87" s="7"/>
-      <c r="D87" s="7"/>
-    </row>
-    <row r="88" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B88" s="7"/>
+    </row>
+    <row r="88" spans="1:6" ht="15.75" customHeight="1">
       <c r="C88" s="7"/>
     </row>
-    <row r="89" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:6" ht="15.75" customHeight="1">
       <c r="C89" s="7"/>
     </row>
-    <row r="90" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:6" ht="15.75" customHeight="1">
       <c r="C90" s="7"/>
     </row>
-    <row r="91" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:6" ht="15.75" customHeight="1">
       <c r="C91" s="7"/>
     </row>
-    <row r="92" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:6" ht="15.75" customHeight="1">
       <c r="C92" s="7"/>
-    </row>
-    <row r="93" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C93" s="7"/>
-    </row>
-    <row r="94" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C94" s="7"/>
-    </row>
-    <row r="95" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C95" s="7"/>
-    </row>
-    <row r="96" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C96" s="7"/>
-    </row>
-    <row r="97" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C97" s="7"/>
-    </row>
-    <row r="98" spans="3:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C98" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
Added project management doc
</commit_message>
<xml_diff>
--- a/data/Blattabacterium/Blattabacterium_genome-data.xlsx
+++ b/data/Blattabacterium/Blattabacterium_genome-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/PostDoc/HGT_pipeline/data/Blattabacterium/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74F289EB-2BE7-3A49-AEFD-352BAE5EDABC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BEC75C4-7C7A-EA43-81B4-AA4EBF7E9D8C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11440" yWindow="1440" windowWidth="17360" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5520" yWindow="1280" windowWidth="17360" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -888,7 +888,8 @@
     <col min="2" max="2" width="21.5" style="2" customWidth="1"/>
     <col min="3" max="3" width="195" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.83203125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="12.6640625" style="2"/>
+    <col min="5" max="5" width="15.5" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="12.6640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1">
@@ -907,7 +908,7 @@
       <c r="E1" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="10" t="s">
         <v>161</v>
       </c>
     </row>
@@ -1826,7 +1827,7 @@
         <v>124</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="15.75" customHeight="1">
@@ -2013,7 +2014,7 @@
         <v>128</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="15.75" customHeight="1">

</xml_diff>